<commit_message>
feat(F-NAR-019): ATOM-DIF.ENE.001-01 Le cerceau sur les flaques
Réécriture vocale example4 : éclat de flaque, énergie vécue.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.ENE.001-01.xlsx
+++ b/stories/arbres/ATOM-DIF.ENE.001-01.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cour d'école après la pluie</t>
+          <t>cour d'école après la pluie, grille, flaque, cerceau jaune, bottes, bac d'eau</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Sarah, Raphaël, papa, maman</t>
+          <t>Chouchou, Raphaël, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sarah veut faire danser le cerceau jaune sur les flaques. Raphaël arrive avec beaucoup d'énergie et le cerceau tremble. Ils jouent, ils attendent, Sarah demande à maman. Le cerceau danse.</t>
+          <t>Une goutte pend sous la grille. Près des bottes, un éclat de flaque brille. Chouchou veut le cerceau, maintenant. Raphaël saute, trop vite. Le cerceau part. Sourire parti. Elle refuse de foncer. Merci vécu. File des balles, il veut passer. Elle s'arrête, il souffle. Ils versent l'eau. Un éclat de flaque tient près des bottes.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un oiseau secoue une branche près du portail. Trois gouttes tombent dans une flaque ronde. La flaque fait des ronds, tout doucement. L'air sent les feuilles mouillées. Le banc de bois est encore sombre. Papa noue la capuche de Sarah. Elle te tient chaud ? Oui, papa. Elle est un peu rêche. Maman frotte une feuille entre ses doigts. Ça sent le jardin, tu vois ? Le jardin, oui. Un cerceau jaune s'appuie contre le mur. Il a une petite goutte sur le bord. Le soleil perce un tout petit nuage. La flaque devient un miroir. En ce moment, Sarah touche le cerceau. Le plastique est froid, un peu mouillé. Je veux le faire danser. Sur les flaques. On y va, tout doucement. Les bottes de Sarah font un bruit mou. Raphaël arrive dans la cour. Ses chaussures tapent le sol. Tap. Tap. Tap. Il saute sur place. Il a de l'énergie, beaucoup. Il bouge tout le temps. C'est son énergie. Ce n'est pas une faute. Raphaël prend le cerceau jaune. Il le fait tourner très vite. Le cerceau tremble près de la flaque. Moi aussi, le cerceau. À tour de rôle, alors. Sarah tend la main. Le cerceau tourne encore. Raphaël ne s'arrête pas. Sarah regarde maman.</t>
+          <t>Une goutte pend sous la grille. Elle tombe dans la flaque, claire et ronde. Elle a fait plouf ! Tu l'as vue, Chouchou ? Oui, papa. La grille goutte, un peu, après la pluie. Ça sent les feuilles, maman. Tes bottes sont mouillées, Chouchou ? Un peu, maman. Près des bottes, un éclat de flaque brille. Il brille, papa. Tu le vois, près des bottes ? Oui, un petit point. Un cerceau jaune s'appuie contre le mur. Le plastique est froid, un peu mouillé. Il est froid, maman. Le cerceau attend contre le mur ? Oui, maman. Un bac d'eau reste près du mur. Le bac est plein. L'eau du bac, Chouchou ? Elle brille aussi. Je veux le cerceau, maintenant ! Sur la flaque ? Oui, tout de suite. Avec tes bottes ? Oui, maman. En ce moment, Chouchou tend la main. Le cerceau glisse un peu, trop lourd. Il est lourd ! Tu le tiens, Chouchou ? Oui, papa. Raphaël arrive dans la cour. Ses chaussures tapent le sol. J'arrive ! Raphaël ! Il saute sur place, trop vite. Le cerceau ! Moi, le cerceau, maintenant ! Raphaël prend le cerceau jaune. Il le fait tourner trop vite. Le cerceau part vers la flaque. Il part ! Oh. Le cerceau tombe dans l'eau. Ça fait un bruit mou. Il est tombé ! L'éclat de flaque tremble, puis tient. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Raphaël, Chouchou ? Oui, papa. Tes mains sont mouillées, Chouchou ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Un oiseau secoue une branche près du portail. Trois gouttes tombent dans une flaque ronde. La flaque fait des ronds, tout doucement. L'air sent les feuilles mouillées. Le banc de bois est encore sombre. Papa noue la capuche de Sarah. Elle te tient chaud ? Oui, papa. Elle est un peu rêche. Maman frotte une feuille entre ses doigts. Ça sent le jardin, tu vois ? Le jardin, oui. Un cerceau jaune s'appuie contre le mur. Il a une petite goutte sur le bord. Le soleil perce un tout petit nuage. La flaque devient un miroir. En ce moment, Sarah touche le cerceau. Le plastique est froid, un peu mouillé. Je veux le faire danser. Sur les flaques. On y va, tout doucement. Les bottes de Sarah font un bruit mou. Raphaël arrive dans la cour. Ses chaussures tapent le sol. Tap. Tap. Tap. Il saute sur place. Il a de l'énergie, beaucoup. Il bouge tout le temps. C'est son énergie. Ce n'est pas une faute. Raphaël prend le cerceau jaune. Il le fait tourner très vite. Le cerceau tremble près de la flaque. Moi aussi, le cerceau. À tour de rôle, alors. Sarah tend la main. Le cerceau tourne encore. Raphaël ne s'arrête pas. Sarah regarde maman.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une goutte pend sous la grille. Elle tombe dans la flaque, claire et ronde. Elle a fait plouf ! Tu l'as vue, Chouchou ? Oui, papa. La grille goutte, un peu, après la pluie. Ça sent les feuilles, maman. Tes bottes sont mouillées, Chouchou ? Un peu, maman. Près des bottes, un &lt;emphasis level="moderate"&gt;éclat de flaque&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, près des bottes ? Oui, un petit point. Un cerceau jaune s'appuie contre le mur. Le plastique est froid, un peu mouillé. Il est froid, maman. Le cerceau attend contre le mur ? Oui, maman. Un bac d'eau reste près du mur. Le bac est plein. L'eau du bac, Chouchou ? Elle brille aussi. Je veux le cerceau, maintenant ! Sur la flaque ? Oui, tout de suite. Avec tes bottes ? Oui, maman. En ce moment, Chouchou tend la main. Le cerceau glisse un peu, trop lourd. Il est lourd ! Tu le tiens, Chouchou ? Oui, papa. Raphaël arrive dans la cour. Ses chaussures tapent le sol. J'arrive ! Raphaël ! Il saute sur place, trop vite. Le cerceau ! Moi, le cerceau, maintenant ! Raphaël prend le cerceau jaune. Il le fait tourner trop vite. Le cerceau part vers la flaque. Il part ! Oh. Le cerceau tombe dans l'eau. Ça fait un bruit mou. Il est tombé ! L'éclat de flaque tremble, puis tient. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Raphaël, Chouchou ? Oui, papa. Tes mains sont mouillées, Chouchou ? Un peu, maman.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Maman laisse Léa dans la cour. Les chaussures tapent le sol. Nino arrive en sautant. Il a beaucoup d'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Il tourne, il s'arrête, il recommence. Léa le regarde. Un enfant dit : il bouge tout le temps. Maman est encore près du portail. Elle dit : beaucoup d'énergie, ce n'est pas une faute. On peut jouer. On peut attendre. On peut demander à un adulte. Léa hoche la tête. La maîtresse sort un cerceau et un sac de balles. Nino prend un cerceau. Il le fait tourner. Léa veut le même jeu. Elle dit : à tour de rôle. Nino pose le cerceau. Il attend son tour. Puis Léa tourne le cerceau. Nino saute sur place, un peu. L'énergie est encore là. Ce n'est pas une faute. Léa dit : maintenant c'est toi. Nino joue. Après, ils font une file pour les balles. Nino a envie d'aller vite. Léa dit : on peut attendre. Nino souffle. Il reste dans la file. La maîtresse donne une balle. Nino la lance dans le panier. Léa lance aussi. Ils jouent. Plus tard, Nino a encore trop d'énergie pour le tapis. Léa va vers la maîtresse. Elle demande à un adulte. La maîtresse dit : Nino, viens marcher avec moi jusqu'au bac. Nino marche. Il pose les mains sur le bac. L'eau est froide. Il se calme un peu. Léa l'attend. Puis ils versent l'eau ensemble. Maman revient à la fin. Léa dit : Nino a de l'énergie. Maman dit : ce n'est pas une faute. Vous avez pu jouer ou attendre. [pause]</t>
+          <t>Une goutte pend sous la grille. Elle tombe dans la flaque, claire et ronde. Elle a fait plouf ! Tu l'as vue, Chouchou ? Oui, papa. La grille goutte, un peu, après la pluie. Ça sent les feuilles, maman. Tes bottes sont mouillées, Chouchou ? Un peu, maman. Près des bottes, un &lt;emphasis&gt;éclat de flaque&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, près des bottes ? Oui, un petit point. Un cerceau jaune s'appuie contre le mur. Le plastique est froid, un peu mouillé. Il est froid, maman. Le cerceau attend contre le mur ? Oui, maman. Un bac d'eau reste près du mur. Le bac est plein. L'eau du bac, Chouchou ? Elle brille aussi. Je veux le cerceau, maintenant ! Sur la flaque ? Oui, tout de suite. Avec tes bottes ? Oui, maman. En ce moment, Chouchou tend la main. Le cerceau glisse un peu, trop lourd. Il est lourd ! Tu le tiens, Chouchou ? Oui, papa. Raphaël arrive dans la cour. Ses chaussures tapent le sol. J'arrive ! Raphaël ! Il saute sur place, trop vite. Le cerceau ! Moi, le cerceau, maintenant ! Raphaël prend le cerceau jaune. Il le fait tourner trop vite. Le cerceau part vers la flaque. Il part ! Oh. Le cerceau tombe dans l'eau. Ça fait un bruit mou. Il est tombé ! L'éclat de flaque tremble, puis tient. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Raphaël, Chouchou ? Oui, papa. Tes mains sont mouillées, Chouchou ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>énergie</t>
+          <t>éclat de flaque</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,48 +1321,69 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_le_cerceau_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un oiseau secoue une branche près du portail.
-narrateur|Trois gouttes tombent dans une flaque ronde.
-narrateur|La flaque fait des ronds, tout doucement.
-narrateur|L'air sent les feuilles mouillées.
-narrateur|Le banc de bois est encore sombre.
-narrateur|Papa noue la capuche de Sarah.
-papa|Elle te tient chaud ?
+          <t>narrateur|Une goutte pend sous la grille.
+narrateur|Elle tombe dans la flaque, claire et ronde.
+enfant-f|Elle a fait plouf !
+papa|Tu l'as vue, Chouchou ?
 enfant-f|Oui, papa.
-enfant-f|Elle est un peu rêche.
-narrateur|Maman frotte une feuille entre ses doigts.
-maman|Ça sent le jardin, tu vois ?
-enfant-f|Le jardin, oui.
+narrateur|La grille goutte, un peu, après la pluie.
+enfant-f|Ça sent les feuilles, maman.
+maman|Tes bottes sont mouillées, Chouchou ?
+enfant-f|Un peu, maman.
+narrateur|Près des bottes, un éclat de flaque brille.
+enfant-f|Il brille, papa.
+papa|Tu le vois, près des bottes ?
+enfant-f|Oui, un petit point.
 narrateur|Un cerceau jaune s'appuie contre le mur.
-narrateur|Il a une petite goutte sur le bord.
-narrateur|Le soleil perce un tout petit nuage.
-narrateur|La flaque devient un miroir.
-narrateur|En ce moment, Sarah touche le cerceau.
 narrateur|Le plastique est froid, un peu mouillé.
-enfant-f|Je veux le faire danser.
-enfant-f|Sur les flaques.
-papa|On y va, tout doucement.
-narrateur|Les bottes de Sarah font un bruit mou.
+enfant-f|Il est froid, maman.
+maman|Le cerceau attend contre le mur ?
+enfant-f|Oui, maman.
+narrateur|Un bac d'eau reste près du mur.
+enfant-f|Le bac est plein.
+papa|L'eau du bac, Chouchou ?
+enfant-f|Elle brille aussi.
+enfant-f|Je veux le cerceau, maintenant !
+papa|Sur la flaque ?
+enfant-f|Oui, tout de suite.
+maman|Avec tes bottes ?
+enfant-f|Oui, maman.
+narrateur|En ce moment, Chouchou tend la main.
+narrateur|Le cerceau glisse un peu, trop lourd.
+enfant-f|Il est lourd !
+papa|Tu le tiens, Chouchou ?
+enfant-f|Oui, papa.
 narrateur|Raphaël arrive dans la cour.
 narrateur|Ses chaussures tapent le sol.
-narrateur|Tap. Tap. Tap.
-narrateur|Il saute sur place.
-narrateur|Il a de l'énergie, beaucoup.
-enfant-f|Il bouge tout le temps.
-maman|C'est son énergie.
-maman|Ce n'est pas une faute.
+copain|J'arrive !
+enfant-f|Raphaël !
+narrateur|Il saute sur place, trop vite.
+copain|Le cerceau !
+enfant-f|Moi, le cerceau, maintenant !
 narrateur|Raphaël prend le cerceau jaune.
-narrateur|Il le fait tourner très vite.
-narrateur|Le cerceau tremble près de la flaque.
-enfant-f|Moi aussi, le cerceau.
-papa|À tour de rôle, alors.
-narrateur|Sarah tend la main.
-narrateur|Le cerceau tourne encore.
-narrateur|Raphaël ne s'arrête pas.
-narrateur|Sarah regarde maman.</t>
+narrateur|Il le fait tourner trop vite.
+narrateur|Le cerceau part vers la flaque.
+enfant-f|Il part !
+copain|Oh.
+narrateur|Le cerceau tombe dans l'eau.
+narrateur|Ça fait un bruit mou.
+enfant-f|Il est tombé !
+narrateur|L'éclat de flaque tremble, puis tient.
+narrateur|Le sourire de Chouchou disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Raphaël, Chouchou ?
+enfant-f|Oui, papa.
+maman|Tes mains sont mouillées, Chouchou ?
+enfant-f|Un peu, maman.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1399,12 +1420,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Raphaël a de l'énergie. Que peut-on faire ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Raphaël a de l'&lt;emphasis level="moderate"&gt;énergie&lt;/emphasis&gt;. Que peut-on faire ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Nino a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Que peut-on faire ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Raphaël a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Que peut-on faire ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1467,7 +1488,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1478,7 +1499,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1493,11 +1514,11 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
@@ -1508,23 +1529,23 @@
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1539,17 +1560,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=raphael_bouge_trop_vite_que_peut_on_faire; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1582,17 +1603,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sarah va vers maman. Maman, on fait quoi ? On joue avec le cerceau. On attend son tour. Tu peux venir me demander. Viens, Raphaël. On marche jusqu'au bac. Ils marchent. Les bottes font encore un bruit mou. Sarah pose les mains sur le bac. L'eau est froide. Raphaël pose les mains aussi. Il souffle. Il se calme un peu. L'énergie est encore là. Ce n'est pas une faute. On attend un peu. Raphaël pose le cerceau. Il attend son tour. C'est à Sarah. Sarah fait tourner le cerceau. Le cerceau danse près des flaques. Il fait un rond jaune sur l'eau. Maintenant c'est toi. Raphaël reprend le cerceau. Il tourne plus doucement. Ils jouent. Puis ils font une file pour les balles. Raphaël a encore envie d'aller vite. On peut attendre. Raphaël souffle. Il reste dans la file. Chacun son tour. Maman donne une balle rouge. Raphaël la lance vers le panier. Sarah lance aussi. Le panier fait un petit toc.</t>
+          <t>Chouchou veut le cerceau, tout de suite. Je le prends, maintenant ! Elle avance trop vite vers Raphaël. Les mots se bousculent dans sa bouche. Attends. Raphaël saute, trop près de l'eau. Oh. Le sourire ne revient pas. Chouchou refuse de foncer. Elle referme les mains. Personne ne parle. Elle observe le cerceau, un instant. Elle écoute la grille qui goutte. Tu veux le cerceau avec Raphaël ? Papa reste à la même hauteur. On va au bac ? On marche jusqu'au bac ? Oui, maman. Viens, Raphaël. J'y vais. Ils marchent vers le bac. Les bottes font un bruit mou. L'eau, papa. Tu poses les mains ? Oui. Chouchou pose les mains sur le bac. L'eau est froide. Raphaël pose les mains aussi. Elle est froide. Il souffle. Merci, Chouchou. Papa a vu les deux, près du bac. L'eau coule un peu, sous les doigts. Elle est froide. Raphaël pose le cerceau, sans se presser. À toi. D'accord. Chouchou fait tourner le cerceau. Le cerceau passe près des flaques. Il tourne ! Oui. Tu le vois, le rond jaune ? Oui, papa. Tes bottes sont au sec ? Un peu, maman. Le ventre de Chouchou se desserre. Les épaules se relèvent un peu. On reste près du bac ? Oui. Tes mains sont froides ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sarah va vers maman. Maman, on fait quoi ? On joue avec le cerceau. On attend son tour. Tu peux venir me demander. Viens, Raphaël. On marche jusqu'au bac. Ils marchent. Les bottes font encore un bruit mou. Sarah pose les mains sur le bac. L'eau est froide. Raphaël pose les mains aussi. Il souffle. Il se calme un peu. L'énergie est encore là. Ce n'est pas une faute. On attend un peu. Raphaël pose le cerceau. Il attend son tour. C'est à Sarah. Sarah fait tourner le cerceau. Le cerceau danse près des flaques. Il fait un rond jaune sur l'eau. Maintenant c'est toi. Raphaël reprend le cerceau. Il tourne plus doucement. Ils jouent. Puis ils font une file pour les balles. Raphaël a encore envie d'aller vite. On peut attendre. Raphaël souffle. Il reste dans la file. Chacun son tour. Maman donne une balle rouge. Raphaël la lance vers le panier. Sarah lance aussi. Le panier fait un petit toc.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Chouchou veut le cerceau, tout de suite. Je le prends, maintenant ! Elle avance trop vite vers Raphaël. Les mots se bousculent dans sa bouche. Attends. Raphaël saute, trop près de l'eau. Oh. Le sourire ne revient pas. Chouchou refuse de foncer. Elle referme les mains. Personne ne parle. Elle observe le cerceau, un instant. Elle écoute la grille qui goutte. Tu veux le cerceau avec Raphaël ? Papa reste à la même hauteur. On va au &lt;emphasis level="moderate"&gt;bac&lt;/emphasis&gt; ? On marche jusqu'au bac ? Oui, maman. Viens, Raphaël. J'y vais. Ils marchent vers le bac. Les bottes font un bruit mou. L'eau, papa. Tu poses les mains ? Oui. Chouchou pose les mains sur le bac. L'eau est froide. Raphaël pose les mains aussi. Elle est froide. Il souffle. Merci, Chouchou. Papa a vu les deux, près du bac. L'eau coule un peu, sous les doigts. Elle est froide. Raphaël pose le cerceau, sans se presser. À toi. D'accord. Chouchou fait tourner le cerceau. Le cerceau passe près des flaques. Il tourne ! Oui. Tu le vois, le rond jaune ? Oui, papa. Tes bottes sont au sec ? Un peu, maman. Le ventre de Chouchou se desserre. Les épaules se relèvent un peu. On reste près du bac ? Oui. Tes mains sont froides ? Un peu, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Nino a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Ce n'est pas une faute. Léa a joué. Elle a su attendre. Elle a demandé à un adulte. [pause]</t>
+          <t>Chouchou veut le cerceau, tout de suite. Je le prends, maintenant ! Elle avance trop vite vers Raphaël. Les mots se bousculent dans sa bouche. Attends. Raphaël saute, trop près de l'eau. Oh. Le sourire ne revient pas. Chouchou refuse de foncer. Elle referme les mains. Personne ne parle. Elle observe le cerceau, un instant. Elle écoute la grille qui goutte. Tu veux le cerceau avec Raphaël ? Papa reste à la même hauteur. On va au &lt;emphasis&gt;bac&lt;/emphasis&gt; ? On marche jusqu'au bac ? Oui, maman. Viens, Raphaël. J'y vais. Ils marchent vers le bac. Les bottes font un bruit mou. L'eau, papa. Tu poses les mains ? Oui. Chouchou pose les mains sur le bac. L'eau est froide. Raphaël pose les mains aussi. Elle est froide. Il souffle. Merci, Chouchou. Papa a vu les deux, près du bac. L'eau coule un peu, sous les doigts. Elle est froide. Raphaël pose le cerceau, sans se presser. À toi. D'accord. Chouchou fait tourner le cerceau. Le cerceau passe près des flaques. Il tourne ! Oui. Tu le vois, le rond jaune ? Oui, papa. Tes bottes sont au sec ? Un peu, maman. Le ventre de Chouchou se desserre. Les épaules se relèvent un peu. On reste près du bac ? Oui. Tes mains sont froides ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1639,7 +1660,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1647,10 +1668,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1673,30 +1694,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>énergie</t>
+          <t>bac</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1705,10 +1726,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1721,48 +1742,62 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_refuse_va_au_bac_avec_lui; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Sarah va vers maman.
-enfant-f|Maman, on fait quoi ?
-maman|On joue avec le cerceau.
-maman|On attend son tour.
-maman|Tu peux venir me demander.
+          <t>narrateur|Chouchou veut le cerceau, tout de suite.
+enfant-f|Je le prends, maintenant !
+narrateur|Elle avance trop vite vers Raphaël.
+narrateur|Les mots se bousculent dans sa bouche.
+copain|Attends.
+narrateur|Raphaël saute, trop près de l'eau.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Chouchou refuse de foncer.
+narrateur|Elle referme les mains.
+narrateur|Personne ne parle.
+narrateur|Elle observe le cerceau, un instant.
+narrateur|Elle écoute la grille qui goutte.
+papa|Tu veux le cerceau avec Raphaël ?
+narrateur|Papa reste à la même hauteur.
+enfant-f|On va au bac ?
+maman|On marche jusqu'au bac ?
+enfant-f|Oui, maman.
 papa|Viens, Raphaël.
-papa|On marche jusqu'au bac.
-narrateur|Ils marchent.
-narrateur|Les bottes font encore un bruit mou.
-narrateur|Sarah pose les mains sur le bac.
+copain|J'y vais.
+narrateur|Ils marchent vers le bac.
+narrateur|Les bottes font un bruit mou.
+enfant-f|L'eau, papa.
+papa|Tu poses les mains ?
+enfant-f|Oui.
+narrateur|Chouchou pose les mains sur le bac.
 narrateur|L'eau est froide.
 narrateur|Raphaël pose les mains aussi.
+copain|Elle est froide.
 narrateur|Il souffle.
-narrateur|Il se calme un peu.
-maman|L'énergie est encore là.
-maman|Ce n'est pas une faute.
-enfant-f|On attend un peu.
-narrateur|Raphaël pose le cerceau.
-narrateur|Il attend son tour.
-papa|C'est à Sarah.
-narrateur|Sarah fait tourner le cerceau.
-narrateur|Le cerceau danse près des flaques.
-narrateur|Il fait un rond jaune sur l'eau.
-enfant-f|Maintenant c'est toi.
-narrateur|Raphaël reprend le cerceau.
-narrateur|Il tourne plus doucement.
-narrateur|Ils jouent.
-narrateur|Puis ils font une file pour les balles.
-narrateur|Raphaël a encore envie d'aller vite.
-enfant-f|On peut attendre.
-narrateur|Raphaël souffle.
-narrateur|Il reste dans la file.
-maman|Chacun son tour.
-narrateur|Maman donne une balle rouge.
-narrateur|Raphaël la lance vers le panier.
-narrateur|Sarah lance aussi.
-narrateur|Le panier fait un petit toc.</t>
+papa|Merci, Chouchou.
+narrateur|Papa a vu les deux, près du bac.
+maman|L'eau coule un peu, sous les doigts.
+enfant-f|Elle est froide.
+narrateur|Raphaël pose le cerceau, sans se presser.
+copain|À toi.
+enfant-f|D'accord.
+narrateur|Chouchou fait tourner le cerceau.
+narrateur|Le cerceau passe près des flaques.
+enfant-f|Il tourne !
+copain|Oui.
+papa|Tu le vois, le rond jaune ?
+enfant-f|Oui, papa.
+maman|Tes bottes sont au sec ?
+enfant-f|Un peu, maman.
+narrateur|Le ventre de Chouchou se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On reste près du bac ?
+enfant-f|Oui.
+maman|Tes mains sont froides ?
+enfant-f|Un peu, maman.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
@@ -1794,17 +1829,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Le soleil touche le cerceau jaune. On range, et on rentre ? Oui, maman. Sarah porte le cerceau. Raphaël porte la balle rouge. Vous vous dites au revoir ? Au revoir, Sarah. Au revoir, Raphaël. La cour redevient calme. La flaque ne tremble plus. Le cerceau a dansé, aujourd'hui. On le pose contre le mur ? Contre le mur. Sarah pose le cerceau. Il s'appuie, tout droit.</t>
+          <t>Maman pose des balles près du bac. Une file, maintenant ! Raphaël veut passer, trop vite. Il saute vers les balles. Moi d'abord ! Chouchou avance les mains, trop vite. Puis elle s'arrête net. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe les balles, un instant. Elle écoute la grille qui goutte. Près des bottes, un éclat de flaque luit. Là, près des bottes. Tu restes, Raphaël ? Raphaël ne dit rien. Il souffle, sans parler. Oui. Il reste derrière elle. Une balle, maman ? La rouge, Chouchou. Chouchou lance vers le panier. Le panier fait un petit toc. À moi. Raphaël lance à son tour. Tu as soufflé, Raphaël ? Un peu. Le bac est plein, Chouchou ? On verse ? Vous versez ensemble ? Oui, papa. Ils versent l'eau du bac. L'eau rejoint la flaque, sans bruit. Elle part. Elle part. Le cerceau a une goutte, Chouchou ? Sur le bord.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Le soleil touche le cerceau jaune. On range, et on rentre ? Oui, maman. Sarah porte le cerceau. Raphaël porte la balle rouge. Vous vous dites au revoir ? Au revoir, Sarah. Au revoir, Raphaël. La cour redevient calme. La flaque ne tremble plus. Le cerceau a dansé, aujourd'hui. On le pose contre le mur ? Contre le mur. Sarah pose le cerceau. Il s'appuie, tout droit.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman pose des balles près du bac. Une file, maintenant ! Raphaël veut passer, trop vite. Il saute vers les balles. Moi d'abord ! Chouchou avance les mains, trop vite. Puis elle s'arrête net. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe les balles, un instant. Elle écoute la grille qui goutte. Près des bottes, un &lt;emphasis level="moderate"&gt;éclat de flaque&lt;/emphasis&gt; luit. Là, près des bottes. Tu restes, Raphaël ? Raphaël ne dit rien. Il souffle, sans parler. Oui. Il reste derrière elle. Une balle, maman ? La rouge, Chouchou. Chouchou lance vers le panier. Le panier fait un petit toc. À moi. Raphaël lance à son tour. Tu as soufflé, Raphaël ? Un peu. Le bac est plein, Chouchou ? On verse ? Vous versez ensemble ? Oui, papa. Ils versent l'eau du bac. L'eau rejoint la flaque, sans bruit. Elle part. Elle part. Le cerceau a une goutte, Chouchou ? Sur le bord.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman prend la &lt;emphasis&gt;main&lt;/emphasis&gt; de Léa. Nino range un cerceau. Ils se disent au revoir. La cour redevient calme. [pause]</t>
+          <t>Maman pose des balles près du bac. Une file, maintenant ! Raphaël veut passer, trop vite. Il saute vers les balles. Moi d'abord ! Chouchou avance les mains, trop vite. Puis elle s'arrête net. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe les balles, un instant. Elle écoute la grille qui goutte. Près des bottes, un &lt;emphasis&gt;éclat de flaque&lt;/emphasis&gt; luit. Là, près des bottes. Tu restes, Raphaël ? Raphaël ne dit rien. Il souffle, sans parler. Oui. Il reste derrière elle. Une balle, maman ? La rouge, Chouchou. Chouchou lance vers le panier. Le panier fait un petit toc. À moi. Raphaël lance à son tour. Tu as soufflé, Raphaël ? Un peu. Le bac est plein, Chouchou ? On verse ? Vous versez ensemble ? Oui, papa. Ils versent l'eau du bac. L'eau rejoint la flaque, sans bruit. Elle part. Elle part. Le cerceau a une goutte, Chouchou ? Sur le bord. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1851,7 +1886,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1859,10 +1894,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.18</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1885,30 +1920,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de flaque</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1917,10 +1952,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1931,24 +1966,55 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_il_souffle_ils_versent; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Le soleil touche le cerceau jaune.
-maman|On range, et on rentre ?
-enfant-f|Oui, maman.
-narrateur|Sarah porte le cerceau.
-narrateur|Raphaël porte la balle rouge.
-papa|Vous vous dites au revoir ?
-enfant-m|Au revoir, Sarah.
-enfant-f|Au revoir, Raphaël.
-narrateur|La cour redevient calme.
-narrateur|La flaque ne tremble plus.
-maman|Le cerceau a dansé, aujourd'hui.
-papa|On le pose contre le mur ?
-enfant-f|Contre le mur.
-narrateur|Sarah pose le cerceau.
-narrateur|Il s'appuie, tout droit.</t>
+          <t>narrateur|Maman pose des balles près du bac.
+enfant-f|Une file, maintenant !
+narrateur|Raphaël veut passer, trop vite.
+narrateur|Il saute vers les balles.
+copain|Moi d'abord !
+narrateur|Chouchou avance les mains, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Chouchou refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe les balles, un instant.
+narrateur|Elle écoute la grille qui goutte.
+narrateur|Près des bottes, un éclat de flaque luit.
+enfant-f|Là, près des bottes.
+enfant-f|Tu restes, Raphaël ?
+narrateur|Raphaël ne dit rien.
+narrateur|Il souffle, sans parler.
+copain|Oui.
+narrateur|Il reste derrière elle.
+enfant-f|Une balle, maman ?
+maman|La rouge, Chouchou.
+narrateur|Chouchou lance vers le panier.
+narrateur|Le panier fait un petit toc.
+copain|À moi.
+narrateur|Raphaël lance à son tour.
+papa|Tu as soufflé, Raphaël ?
+copain|Un peu.
+maman|Le bac est plein, Chouchou ?
+enfant-f|On verse ?
+papa|Vous versez ensemble ?
+enfant-f|Oui, papa.
+narrateur|Ils versent l'eau du bac.
+narrateur|L'eau rejoint la flaque, sans bruit.
+enfant-f|Elle part.
+copain|Elle part.
+maman|Le cerceau a une goutte, Chouchou ?
+enfant-f|Sur le bord.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>enfants_parc</t>
         </is>
       </c>
     </row>
@@ -1975,17 +2041,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le cerceau jaune sèche un peu. Il a encore une goutte sur le bord. Il attend demain. Sur les flaques.</t>
+          <t>Ils restent près de la flaque. Maman essuie un peu d'eau. On a versé l'eau, papa. Tu l'as vue, toi ? Oui, dans la flaque. On est bien, ici. Chouchou tapote le cerceau du doigt. Il a une goutte, maman. Tu la vois, la goutte ? Oui, maman. Le cerceau est resté, Chouchou. Oui, avec Raphaël. Le cerceau est resté. Ça sent la pluie, un peu tiède. Et la grille, maman. Oui, dans l'air. Les bottes restent près de l'eau. Un éclat de flaque tient près des bottes.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le cerceau jaune sèche un peu. Il a encore une goutte sur le bord. Il attend demain. Sur les flaques.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la flaque. Maman essuie un peu d'eau. On a versé l'eau, papa. Tu l'as vue, toi ? Oui, dans la flaque. On est bien, ici. Chouchou tapote le cerceau du doigt. Il a une goutte, maman. Tu la vois, la goutte ? Oui, maman. Le cerceau est resté, Chouchou. Oui, avec Raphaël. Le cerceau est resté. Ça sent la pluie, un peu tiède. Et la grille, maman. Oui, dans l'air. Les bottes restent près de l'eau. Un &lt;emphasis level="moderate"&gt;éclat de flaque&lt;/emphasis&gt; tient près des bottes.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la flaque. Maman essuie un peu d'eau. On a versé l'eau, papa. Tu l'as vue, toi ? Oui, dans la flaque. On est bien, ici. Chouchou tapote le cerceau du doigt. Il a une goutte, maman. Tu la vois, la goutte ? Oui, maman. Le cerceau est resté, Chouchou. Oui, avec Raphaël. Le cerceau est resté. Ça sent la pluie, un peu tiède. Et la grille, maman. Oui, dans l'air. Les bottes restent près de l'eau. Un &lt;emphasis&gt;éclat de flaque&lt;/emphasis&gt; tient près des bottes.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2032,7 +2098,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2040,10 +2106,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2052,12 +2118,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2066,17 +2132,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de flaque</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2085,11 +2155,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2098,27 +2168,45 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_pres_des_bottes; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le cerceau jaune sèche un peu.
-narrateur|Il a encore une goutte sur le bord.
-papa|Il attend demain.
-enfant-f|Sur les flaques.</t>
+          <t>narrateur|Ils restent près de la flaque.
+narrateur|Maman essuie un peu d'eau.
+enfant-f|On a versé l'eau, papa.
+papa|Tu l'as vue, toi ?
+enfant-f|Oui, dans la flaque.
+maman|On est bien, ici.
+narrateur|Chouchou tapote le cerceau du doigt.
+enfant-f|Il a une goutte, maman.
+maman|Tu la vois, la goutte ?
+enfant-f|Oui, maman.
+papa|Le cerceau est resté, Chouchou.
+enfant-f|Oui, avec Raphaël.
+copain|Le cerceau est resté.
+narrateur|Ça sent la pluie, un peu tiède.
+enfant-f|Et la grille, maman.
+maman|Oui, dans l'air.
+narrateur|Les bottes restent près de l'eau.
+narrateur|Un éclat de flaque tient près des bottes.</t>
         </is>
       </c>
     </row>
@@ -2139,7 +2227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2224,6 +2312,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>